<commit_message>
Publish yassir + caribbean economics sheets; Tasklet image asset brief
Register LB-83 sheet IDs, build/upload transparent workbooks, wire economics_url
into partner JSON and deck configs. Document why adani/reliance remain held-null
(no finance engine rows). Add Tasklet note for deck-studio N30/background assets.
</commit_message>
<xml_diff>
--- a/finance/_sheet_out/yassir_unit_econ.xlsx
+++ b/finance/_sheet_out/yassir_unit_econ.xlsx
@@ -44,9 +44,9 @@
     <definedName name="scenario">'Assumptions'!$B$35</definedName>
     <definedName name="load_sel">'Assumptions'!$B$36</definedName>
     <definedName name="revleg_sel">'Assumptions'!$B$37</definedName>
-    <definedName name="country_opex">'Country opex'!$A$4:$G$5</definedName>
-    <definedName name="som_floor_fleet">'Corridor economics'!$D$25</definedName>
-    <definedName name="som_floor_rev">'Corridor economics'!$E$25</definedName>
+    <definedName name="country_opex">'Country opex'!$A$4:$G$6</definedName>
+    <definedName name="som_floor_fleet">'Corridor economics'!$D$27</definedName>
+    <definedName name="som_floor_rev">'Corridor economics'!$E$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1708,7 +1708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1773,58 +1773,88 @@
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="B4" s="26" t="n">
-        <v>14000</v>
+        <v>12000</v>
       </c>
       <c r="C4" s="27" t="n">
-        <v>0.12</v>
+        <v>0.04</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>0.38</v>
+        <v>0.3</v>
       </c>
       <c r="G4" s="26" t="n">
         <v>600000</v>
       </c>
       <c r="H4" s="14" t="inlineStr">
         <is>
-          <t>Modeled from national maritime-wage / cost-of-living index vs SG anchor | Modeled from national commercial electricity tariff avg | Modeled berth/marina overhead vs SG anchor by cost index | CAPEX LB-243 US/EU=$900K else $600K</t>
+          <t>Regional modeled maritime-wage proxy retained because no strong Algeria maritime-captain salary source was found; acceptable only as labelled draft until local wage source replaces it. | GlobalPetrolPrices Algeria electricity page reports September 2025 business electricity at USD 0.035/kWh, citing CREG, Ministry of Energy and Mines, and Sonelgaz; rounded up to 0.04/kWh for operating conservatism. | Regional modeled marina/port overhead proxy retained; Algeria marina-fee search found weak port/marina leads but no tariff table. Replace before final investment-grade economics if available. | CAPEX LB-243 US/EU=$900K else $600K</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B5" s="26" t="n">
         <v>14000</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.45</v>
+        <v>0.6</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>9000</v>
+        <v>10000</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="G5" s="26" t="n">
         <v>600000</v>
       </c>
       <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>Modeled from national maritime-wage / cost-of-living index vs SG anchor | Modeled from national commercial electricity tariff avg | Modeled berth/marina overhead vs SG anchor by cost index | CAPEX LB-243 US/EU=$900K else $600K</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="n">
+        <v>14000</v>
+      </c>
+      <c r="C6" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E6" s="26" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G6" s="26" t="n">
+        <v>600000</v>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>Modeled from national maritime-wage / cost-of-living index vs SG anchor | Modeled from national commercial electricity tariff avg | Modeled berth/marina overhead vs SG anchor by cost index | CAPEX LB-243 US/EU=$900K else $600K</t>
         </is>
@@ -1844,7 +1874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX28"/>
+  <dimension ref="A1:AX32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2175,23 +2205,25 @@
     <row r="4">
       <c r="A4" s="29" t="inlineStr">
         <is>
-          <t>Yassir Morocco</t>
+          <t>Yassir Algeria</t>
         </is>
       </c>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="C4" s="30" t="inlineStr">
         <is>
-          <t>Rabat → Sale</t>
+          <t>La Pêcherie / Port d'Alger → El Djamila / Aïn Bénian</t>
         </is>
       </c>
       <c r="D4" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E4" s="26" t="n"/>
+        <v>8.5</v>
+      </c>
+      <c r="E4" s="26" t="n">
+        <v>18</v>
+      </c>
       <c r="F4" s="32" t="n"/>
       <c r="G4" s="32" t="n"/>
       <c r="H4" s="19" t="n">
@@ -2206,7 +2238,7 @@
         <v/>
       </c>
       <c r="K4" s="34">
-        <f>MIN(16,FLOOR(60*service_hr/J4,1))</f>
+        <f>MIN(10,FLOOR(60*service_hr/J4,1))</f>
         <v/>
       </c>
       <c r="L4" s="34">
@@ -2293,7 +2325,9 @@
         <f>((D4*O4/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D4*O4*VLOOKUP(B4,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG4" s="31" t="n"/>
+      <c r="AG4" s="31" t="n">
+        <v>170280</v>
+      </c>
       <c r="AH4" s="32" t="n"/>
       <c r="AI4" s="32" t="n"/>
       <c r="AJ4" s="39" t="n">
@@ -2335,7 +2369,11 @@
         <f>IF(((S4*pax_cap*load_full*ROUND(K4*L4*revleg_full,0))-(((battery/range_nm)*D4*ROUND(K4*L4*revleg_full,0)*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4))&lt;=0,"",VLOOKUP(B4,country_opex,7,FALSE)/((S4*pax_cap*load_full*ROUND(K4*L4*revleg_full,0))-(((battery/range_nm)*D4*ROUND(K4*L4*revleg_full,0)*VLOOKUP(B4,country_opex,3,FALSE))+V4+W4+X4+Y4+Z4)))</f>
         <v/>
       </c>
-      <c r="AW4" s="44" t="n"/>
+      <c r="AW4" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[LB-255 PREMIUM RE-FARE: subsidized comparable $3.7 lifted to premium on-demand floor $18.0] </t>
+        </is>
+      </c>
       <c r="AX4" s="44" t="n"/>
     </row>
     <row r="5">
@@ -2351,25 +2389,15 @@
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Tangier Marina Bay → Tarifa (cross-strait excluded)</t>
+          <t>Rabat → Sale</t>
         </is>
       </c>
       <c r="D5" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" s="26" t="n">
-        <v>43.5</v>
-      </c>
-      <c r="F5" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G5" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="E5" s="26" t="n"/>
+      <c r="F5" s="32" t="n"/>
+      <c r="G5" s="32" t="n"/>
       <c r="H5" s="19" t="n">
         <v>1</v>
       </c>
@@ -2382,7 +2410,7 @@
         <v/>
       </c>
       <c r="K5" s="34">
-        <f>MIN(10,FLOOR(60*service_hr/J5,1))</f>
+        <f>MIN(16,FLOOR(60*service_hr/J5,1))</f>
         <v/>
       </c>
       <c r="L5" s="34">
@@ -2469,9 +2497,7 @@
         <f>((D5*O5/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D5*O5*VLOOKUP(B5,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG5" s="31" t="n">
-        <v>760778</v>
-      </c>
+      <c r="AG5" s="31" t="n"/>
       <c r="AH5" s="32" t="n"/>
       <c r="AI5" s="32" t="n"/>
       <c r="AJ5" s="39" t="n">
@@ -2513,11 +2539,7 @@
         <f>IF(((S5*pax_cap*load_full*ROUND(K5*L5*revleg_full,0))-(((battery/range_nm)*D5*ROUND(K5*L5*revleg_full,0)*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5))&lt;=0,"",VLOOKUP(B5,country_opex,7,FALSE)/((S5*pax_cap*load_full*ROUND(K5*L5*revleg_full,0))-(((battery/range_nm)*D5*ROUND(K5*L5*revleg_full,0)*VLOOKUP(B5,country_opex,3,FALSE))+V5+W5+X5+Y5+Z5)))</f>
         <v/>
       </c>
-      <c r="AW5" s="44" t="inlineStr">
-        <is>
-          <t>PREMIUM tier: standard adult FOOT-PASSENGER one-way fast-ferry fare Tarifa&lt;-&gt;Tangier Ville ~EUR 40.25 (traveller-reported foot fare) x 1.08 = ~$43.5; DirectFerries lists 'from $46'. THIS is the Navier-modeled per-seat tier.</t>
-        </is>
-      </c>
+      <c r="AW5" s="44" t="n"/>
       <c r="AX5" s="44" t="n"/>
     </row>
     <row r="6">
@@ -2533,15 +2555,25 @@
       </c>
       <c r="C6" s="30" t="inlineStr">
         <is>
-          <t>Agadir Marina → Taghazout</t>
+          <t>Tangier Marina Bay → Tarifa (cross-strait excluded)</t>
         </is>
       </c>
       <c r="D6" s="31" t="n">
-        <v>9</v>
-      </c>
-      <c r="E6" s="26" t="n"/>
-      <c r="F6" s="32" t="n"/>
-      <c r="G6" s="32" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="E6" s="26" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="F6" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G6" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H6" s="19" t="n">
         <v>1</v>
       </c>
@@ -2642,7 +2674,7 @@
         <v/>
       </c>
       <c r="AG6" s="31" t="n">
-        <v>77500</v>
+        <v>760778</v>
       </c>
       <c r="AH6" s="32" t="n"/>
       <c r="AI6" s="32" t="n"/>
@@ -2685,7 +2717,11 @@
         <f>IF(((S6*pax_cap*load_full*ROUND(K6*L6*revleg_full,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_full,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6))&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/((S6*pax_cap*load_full*ROUND(K6*L6*revleg_full,0))-(((battery/range_nm)*D6*ROUND(K6*L6*revleg_full,0)*VLOOKUP(B6,country_opex,3,FALSE))+V6+W6+X6+Y6+Z6)))</f>
         <v/>
       </c>
-      <c r="AW6" s="44" t="n"/>
+      <c r="AW6" s="44" t="inlineStr">
+        <is>
+          <t>PREMIUM tier: standard adult FOOT-PASSENGER one-way fast-ferry fare Tarifa&lt;-&gt;Tangier Ville ~EUR 40.25 (traveller-reported foot fare) x 1.08 = ~$43.5; DirectFerries lists 'from $46'. THIS is the Navier-modeled per-seat tier.</t>
+        </is>
+      </c>
       <c r="AX6" s="44" t="n"/>
     </row>
     <row r="7">
@@ -2701,25 +2737,15 @@
       </c>
       <c r="C7" s="30" t="inlineStr">
         <is>
-          <t>Tanger Med (Ksar el Majaz) → Algeciras (Spain)</t>
+          <t>Agadir Marina → Taghazout</t>
         </is>
       </c>
       <c r="D7" s="31" t="n">
-        <v>13</v>
-      </c>
-      <c r="E7" s="26" t="n">
-        <v>38</v>
-      </c>
-      <c r="F7" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G7" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="E7" s="26" t="n"/>
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="n"/>
       <c r="H7" s="19" t="n">
         <v>1</v>
       </c>
@@ -2820,7 +2846,7 @@
         <v/>
       </c>
       <c r="AG7" s="31" t="n">
-        <v>1610211</v>
+        <v>77500</v>
       </c>
       <c r="AH7" s="32" t="n"/>
       <c r="AI7" s="32" t="n"/>
@@ -2863,11 +2889,7 @@
         <f>IF(((S7*pax_cap*load_full*ROUND(K7*L7*revleg_full,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_full,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7))&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/((S7*pax_cap*load_full*ROUND(K7*L7*revleg_full,0))-(((battery/range_nm)*D7*ROUND(K7*L7*revleg_full,0)*VLOOKUP(B7,country_opex,3,FALSE))+V7+W7+X7+Y7+Z7)))</f>
         <v/>
       </c>
-      <c r="AW7" s="44" t="inlineStr">
-        <is>
-          <t>PREMIUM tier: standard adult FOOT-PASSENGER one-way Tanger Med&lt;-&gt;Algeciras ~EUR 35 x 1.08 = ~$38 (Strait fast-ferry foot fares cluster EUR 30-40).</t>
-        </is>
-      </c>
+      <c r="AW7" s="44" t="n"/>
       <c r="AX7" s="44" t="n"/>
     </row>
     <row r="8">
@@ -2883,15 +2905,25 @@
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>Casablanca → Mohammedia</t>
+          <t>Tanger Med (Ksar el Majaz) → Algeciras (Spain)</t>
         </is>
       </c>
       <c r="D8" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="E8" s="26" t="n"/>
-      <c r="F8" s="32" t="n"/>
-      <c r="G8" s="32" t="n"/>
+      <c r="E8" s="26" t="n">
+        <v>38</v>
+      </c>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G8" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H8" s="19" t="n">
         <v>1</v>
       </c>
@@ -2904,7 +2936,7 @@
         <v/>
       </c>
       <c r="K8" s="34">
-        <f>MIN(16,FLOOR(60*service_hr/J8,1))</f>
+        <f>MIN(10,FLOOR(60*service_hr/J8,1))</f>
         <v/>
       </c>
       <c r="L8" s="34">
@@ -2991,7 +3023,9 @@
         <f>((D8*O8/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D8*O8*VLOOKUP(B8,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG8" s="31" t="n"/>
+      <c r="AG8" s="31" t="n">
+        <v>1610211</v>
+      </c>
       <c r="AH8" s="32" t="n"/>
       <c r="AI8" s="32" t="n"/>
       <c r="AJ8" s="39" t="n">
@@ -3033,7 +3067,11 @@
         <f>IF(((S8*pax_cap*load_full*ROUND(K8*L8*revleg_full,0))-(((battery/range_nm)*D8*ROUND(K8*L8*revleg_full,0)*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8))&lt;=0,"",VLOOKUP(B8,country_opex,7,FALSE)/((S8*pax_cap*load_full*ROUND(K8*L8*revleg_full,0))-(((battery/range_nm)*D8*ROUND(K8*L8*revleg_full,0)*VLOOKUP(B8,country_opex,3,FALSE))+V8+W8+X8+Y8+Z8)))</f>
         <v/>
       </c>
-      <c r="AW8" s="44" t="n"/>
+      <c r="AW8" s="44" t="inlineStr">
+        <is>
+          <t>PREMIUM tier: standard adult FOOT-PASSENGER one-way Tanger Med&lt;-&gt;Algeciras ~EUR 35 x 1.08 = ~$38 (Strait fast-ferry foot fares cluster EUR 30-40).</t>
+        </is>
+      </c>
       <c r="AX8" s="44" t="n"/>
     </row>
     <row r="9">
@@ -3049,11 +3087,11 @@
       </c>
       <c r="C9" s="30" t="inlineStr">
         <is>
-          <t>Al Hoceima → Cala Iris</t>
+          <t>Casablanca → Mohammedia</t>
         </is>
       </c>
       <c r="D9" s="31" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E9" s="26" t="n"/>
       <c r="F9" s="32" t="n"/>
@@ -3215,25 +3253,15 @@
       </c>
       <c r="C10" s="30" t="inlineStr">
         <is>
-          <t>Tanger Med → Ceuta (Spanish enclave)</t>
+          <t>Al Hoceima → Cala Iris</t>
         </is>
       </c>
       <c r="D10" s="31" t="n">
-        <v>22</v>
-      </c>
-      <c r="E10" s="26" t="n">
-        <v>36</v>
-      </c>
-      <c r="F10" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G10" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="E10" s="26" t="n"/>
+      <c r="F10" s="32" t="n"/>
+      <c r="G10" s="32" t="n"/>
       <c r="H10" s="19" t="n">
         <v>1</v>
       </c>
@@ -3246,7 +3274,7 @@
         <v/>
       </c>
       <c r="K10" s="34">
-        <f>MIN(10,FLOOR(60*service_hr/J10,1))</f>
+        <f>MIN(16,FLOOR(60*service_hr/J10,1))</f>
         <v/>
       </c>
       <c r="L10" s="34">
@@ -3375,11 +3403,7 @@
         <f>IF(((S10*pax_cap*load_full*ROUND(K10*L10*revleg_full,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_full,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10))&lt;=0,"",VLOOKUP(B10,country_opex,7,FALSE)/((S10*pax_cap*load_full*ROUND(K10*L10*revleg_full,0))-(((battery/range_nm)*D10*ROUND(K10*L10*revleg_full,0)*VLOOKUP(B10,country_opex,3,FALSE))+V10+W10+X10+Y10+Z10)))</f>
         <v/>
       </c>
-      <c r="AW10" s="44" t="inlineStr">
-        <is>
-          <t>PREMIUM tier (nearest comparable = Algeciras&lt;-&gt;Ceuta fast ferry): avg foot-passenger fare ~EUR 33 x 1.08 ~= $36 (one-way ~EUR 25-35), 60 min fast ferry.</t>
-        </is>
-      </c>
+      <c r="AW10" s="44" t="n"/>
       <c r="AX10" s="44" t="n"/>
     </row>
     <row r="11">
@@ -3395,15 +3419,25 @@
       </c>
       <c r="C11" s="30" t="inlineStr">
         <is>
-          <t>Casablanca → Rabat</t>
+          <t>Tanger Med → Ceuta (Spanish enclave)</t>
         </is>
       </c>
       <c r="D11" s="31" t="n">
-        <v>46</v>
-      </c>
-      <c r="E11" s="26" t="n"/>
-      <c r="F11" s="32" t="n"/>
-      <c r="G11" s="32" t="n"/>
+        <v>22</v>
+      </c>
+      <c r="E11" s="26" t="n">
+        <v>36</v>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H11" s="19" t="n">
         <v>1</v>
       </c>
@@ -3416,7 +3450,7 @@
         <v/>
       </c>
       <c r="K11" s="34">
-        <f>MIN(16,FLOOR(60*service_hr/J11,1))</f>
+        <f>MIN(10,FLOOR(60*service_hr/J11,1))</f>
         <v/>
       </c>
       <c r="L11" s="34">
@@ -3503,9 +3537,7 @@
         <f>((D11*O11/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D11*O11*VLOOKUP(B11,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG11" s="31" t="n">
-        <v>165000</v>
-      </c>
+      <c r="AG11" s="31" t="n"/>
       <c r="AH11" s="32" t="n"/>
       <c r="AI11" s="32" t="n"/>
       <c r="AJ11" s="39" t="n">
@@ -3547,27 +3579,31 @@
         <f>IF(((S11*pax_cap*load_full*ROUND(K11*L11*revleg_full,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_full,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11))&lt;=0,"",VLOOKUP(B11,country_opex,7,FALSE)/((S11*pax_cap*load_full*ROUND(K11*L11*revleg_full,0))-(((battery/range_nm)*D11*ROUND(K11*L11*revleg_full,0)*VLOOKUP(B11,country_opex,3,FALSE))+V11+W11+X11+Y11+Z11)))</f>
         <v/>
       </c>
-      <c r="AW11" s="44" t="n"/>
+      <c r="AW11" s="44" t="inlineStr">
+        <is>
+          <t>PREMIUM tier (nearest comparable = Algeciras&lt;-&gt;Ceuta fast ferry): avg foot-passenger fare ~EUR 33 x 1.08 ~= $36 (one-way ~EUR 25-35), 60 min fast ferry.</t>
+        </is>
+      </c>
       <c r="AX11" s="44" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
-          <t>Yassir Tunisia</t>
+          <t>Yassir Morocco</t>
         </is>
       </c>
       <c r="B12" s="29" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="C12" s="30" t="inlineStr">
         <is>
-          <t>Jorf (mainland) → Ajim (Djerba Island)</t>
+          <t>Casablanca → Rabat</t>
         </is>
       </c>
       <c r="D12" s="31" t="n">
-        <v>1.1</v>
+        <v>46</v>
       </c>
       <c r="E12" s="26" t="n"/>
       <c r="F12" s="32" t="n"/>
@@ -3584,7 +3620,7 @@
         <v/>
       </c>
       <c r="K12" s="34">
-        <f>MIN(10,FLOOR(60*service_hr/J12,1))</f>
+        <f>MIN(16,FLOOR(60*service_hr/J12,1))</f>
         <v/>
       </c>
       <c r="L12" s="34">
@@ -3672,7 +3708,7 @@
         <v/>
       </c>
       <c r="AG12" s="31" t="n">
-        <v>2463750</v>
+        <v>165000</v>
       </c>
       <c r="AH12" s="32" t="n"/>
       <c r="AI12" s="32" t="n"/>
@@ -3731,25 +3767,15 @@
       </c>
       <c r="C13" s="30" t="inlineStr">
         <is>
-          <t>La Goulette → Sidi Bou Said</t>
+          <t>Jorf (mainland) → Ajim (Djerba Island)</t>
         </is>
       </c>
       <c r="D13" s="31" t="n">
-        <v>4</v>
-      </c>
-      <c r="E13" s="26" t="n">
-        <v>27</v>
-      </c>
-      <c r="F13" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G13" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>1.1</v>
+      </c>
+      <c r="E13" s="26" t="n"/>
+      <c r="F13" s="32" t="n"/>
+      <c r="G13" s="32" t="n"/>
       <c r="H13" s="19" t="n">
         <v>1</v>
       </c>
@@ -3850,7 +3876,7 @@
         <v/>
       </c>
       <c r="AG13" s="31" t="n">
-        <v>222000</v>
+        <v>2463750</v>
       </c>
       <c r="AH13" s="32" t="n"/>
       <c r="AI13" s="32" t="n"/>
@@ -3893,11 +3919,7 @@
         <f>IF(((S13*pax_cap*load_full*ROUND(K13*L13*revleg_full,0))-(((battery/range_nm)*D13*ROUND(K13*L13*revleg_full,0)*VLOOKUP(B13,country_opex,3,FALSE))+V13+W13+X13+Y13+Z13))&lt;=0,"",VLOOKUP(B13,country_opex,7,FALSE)/((S13*pax_cap*load_full*ROUND(K13*L13*revleg_full,0))-(((battery/range_nm)*D13*ROUND(K13*L13*revleg_full,0)*VLOOKUP(B13,country_opex,3,FALSE))+V13+W13+X13+Y13+Z13)))</f>
         <v/>
       </c>
-      <c r="AW13" s="44" t="inlineStr">
-        <is>
-          <t>PREMIUM charter-divided tier: Gulf of Tunis / Sidi Bou Said per-seat excursion cruise ~EUR 25 (pirate-boat dinner cruise 'from EUR 30'; 3h marina cruise EUR 15-20) x 1.08 ~= $27. Nearest premium per-seat water product on this corridor; no scheduled fast catamaran exists.</t>
-        </is>
-      </c>
+      <c r="AW13" s="44" t="n"/>
       <c r="AX13" s="44" t="n"/>
     </row>
     <row r="14">
@@ -3913,15 +3935,25 @@
       </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Tunis (Tunis Marine) → La Goulette</t>
+          <t>La Goulette → Sidi Bou Said</t>
         </is>
       </c>
       <c r="D14" s="31" t="n">
-        <v>5</v>
-      </c>
-      <c r="E14" s="26" t="n"/>
-      <c r="F14" s="32" t="n"/>
-      <c r="G14" s="32" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="E14" s="26" t="n">
+        <v>27</v>
+      </c>
+      <c r="F14" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G14" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H14" s="19" t="n">
         <v>1</v>
       </c>
@@ -3934,7 +3966,7 @@
         <v/>
       </c>
       <c r="K14" s="34">
-        <f>MIN(16,FLOOR(60*service_hr/J14,1))</f>
+        <f>MIN(10,FLOOR(60*service_hr/J14,1))</f>
         <v/>
       </c>
       <c r="L14" s="34">
@@ -4022,7 +4054,7 @@
         <v/>
       </c>
       <c r="AG14" s="31" t="n">
-        <v>296000</v>
+        <v>222000</v>
       </c>
       <c r="AH14" s="32" t="n"/>
       <c r="AI14" s="32" t="n"/>
@@ -4065,7 +4097,11 @@
         <f>IF(((S14*pax_cap*load_full*ROUND(K14*L14*revleg_full,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_full,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14))&lt;=0,"",VLOOKUP(B14,country_opex,7,FALSE)/((S14*pax_cap*load_full*ROUND(K14*L14*revleg_full,0))-(((battery/range_nm)*D14*ROUND(K14*L14*revleg_full,0)*VLOOKUP(B14,country_opex,3,FALSE))+V14+W14+X14+Y14+Z14)))</f>
         <v/>
       </c>
-      <c r="AW14" s="44" t="n"/>
+      <c r="AW14" s="44" t="inlineStr">
+        <is>
+          <t>PREMIUM charter-divided tier: Gulf of Tunis / Sidi Bou Said per-seat excursion cruise ~EUR 25 (pirate-boat dinner cruise 'from EUR 30'; 3h marina cruise EUR 15-20) x 1.08 ~= $27. Nearest premium per-seat water product on this corridor; no scheduled fast catamaran exists.</t>
+        </is>
+      </c>
       <c r="AX14" s="44" t="n"/>
     </row>
     <row r="15">
@@ -4081,11 +4117,11 @@
       </c>
       <c r="C15" s="30" t="inlineStr">
         <is>
-          <t>Tunis (La Goulette) → La Marsa / Gammarth</t>
+          <t>Tunis (Tunis Marine) → La Goulette</t>
         </is>
       </c>
       <c r="D15" s="31" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E15" s="26" t="n"/>
       <c r="F15" s="32" t="n"/>
@@ -4190,7 +4226,7 @@
         <v/>
       </c>
       <c r="AG15" s="31" t="n">
-        <v>222000</v>
+        <v>296000</v>
       </c>
       <c r="AH15" s="32" t="n"/>
       <c r="AI15" s="32" t="n"/>
@@ -4249,25 +4285,15 @@
       </c>
       <c r="C16" s="30" t="inlineStr">
         <is>
-          <t>Yasmine Hammamet → Nabeul</t>
+          <t>Tunis (La Goulette) → La Marsa / Gammarth</t>
         </is>
       </c>
       <c r="D16" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="E16" s="26" t="n">
-        <v>22</v>
-      </c>
-      <c r="F16" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G16" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+      <c r="E16" s="26" t="n"/>
+      <c r="F16" s="32" t="n"/>
+      <c r="G16" s="32" t="n"/>
       <c r="H16" s="19" t="n">
         <v>1</v>
       </c>
@@ -4280,7 +4306,7 @@
         <v/>
       </c>
       <c r="K16" s="34">
-        <f>MIN(10,FLOOR(60*service_hr/J16,1))</f>
+        <f>MIN(16,FLOOR(60*service_hr/J16,1))</f>
         <v/>
       </c>
       <c r="L16" s="34">
@@ -4367,7 +4393,9 @@
         <f>((D16*O16/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D16*O16*VLOOKUP(B16,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG16" s="31" t="n"/>
+      <c r="AG16" s="31" t="n">
+        <v>222000</v>
+      </c>
       <c r="AH16" s="32" t="n"/>
       <c r="AI16" s="32" t="n"/>
       <c r="AJ16" s="39" t="n">
@@ -4409,11 +4437,7 @@
         <f>IF(((S16*pax_cap*load_full*ROUND(K16*L16*revleg_full,0))-(((battery/range_nm)*D16*ROUND(K16*L16*revleg_full,0)*VLOOKUP(B16,country_opex,3,FALSE))+V16+W16+X16+Y16+Z16))&lt;=0,"",VLOOKUP(B16,country_opex,7,FALSE)/((S16*pax_cap*load_full*ROUND(K16*L16*revleg_full,0))-(((battery/range_nm)*D16*ROUND(K16*L16*revleg_full,0)*VLOOKUP(B16,country_opex,3,FALSE))+V16+W16+X16+Y16+Z16)))</f>
         <v/>
       </c>
-      <c r="AW16" s="44" t="inlineStr">
-        <is>
-          <t>PREMIUM charter-divided tier: Hammamet/Nabeul bay per-seat excursion boat ~EUR 15-25 (3h marina cruise w/ swim stop) -&gt; ~EUR 20 x 1.08 ~= $22. Nearest premium per-seat water product on the bay.</t>
-        </is>
-      </c>
+      <c r="AW16" s="44" t="n"/>
       <c r="AX16" s="44" t="n"/>
     </row>
     <row r="17">
@@ -4429,15 +4453,25 @@
       </c>
       <c r="C17" s="30" t="inlineStr">
         <is>
-          <t>Sfax → Sidi Youssef (Kerkennah Islands)</t>
+          <t>Yasmine Hammamet → Nabeul</t>
         </is>
       </c>
       <c r="D17" s="31" t="n">
-        <v>11</v>
-      </c>
-      <c r="E17" s="26" t="n"/>
-      <c r="F17" s="32" t="n"/>
-      <c r="G17" s="32" t="n"/>
+        <v>7</v>
+      </c>
+      <c r="E17" s="26" t="n">
+        <v>22</v>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G17" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H17" s="19" t="n">
         <v>1</v>
       </c>
@@ -4537,9 +4571,7 @@
         <f>((D17*O17/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D17*O17*VLOOKUP(B17,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG17" s="31" t="n">
-        <v>1750000</v>
-      </c>
+      <c r="AG17" s="31" t="n"/>
       <c r="AH17" s="32" t="n"/>
       <c r="AI17" s="32" t="n"/>
       <c r="AJ17" s="39" t="n">
@@ -4581,7 +4613,11 @@
         <f>IF(((S17*pax_cap*load_full*ROUND(K17*L17*revleg_full,0))-(((battery/range_nm)*D17*ROUND(K17*L17*revleg_full,0)*VLOOKUP(B17,country_opex,3,FALSE))+V17+W17+X17+Y17+Z17))&lt;=0,"",VLOOKUP(B17,country_opex,7,FALSE)/((S17*pax_cap*load_full*ROUND(K17*L17*revleg_full,0))-(((battery/range_nm)*D17*ROUND(K17*L17*revleg_full,0)*VLOOKUP(B17,country_opex,3,FALSE))+V17+W17+X17+Y17+Z17)))</f>
         <v/>
       </c>
-      <c r="AW17" s="44" t="n"/>
+      <c r="AW17" s="44" t="inlineStr">
+        <is>
+          <t>PREMIUM charter-divided tier: Hammamet/Nabeul bay per-seat excursion boat ~EUR 15-25 (3h marina cruise w/ swim stop) -&gt; ~EUR 20 x 1.08 ~= $22. Nearest premium per-seat water product on the bay.</t>
+        </is>
+      </c>
       <c r="AX17" s="44" t="n"/>
     </row>
     <row r="18">
@@ -4597,25 +4633,15 @@
       </c>
       <c r="C18" s="30" t="inlineStr">
         <is>
-          <t>Sousse (Port El Kantaoui) → Monastir (Marina)</t>
+          <t>Sfax → Sidi Youssef (Kerkennah Islands)</t>
         </is>
       </c>
       <c r="D18" s="31" t="n">
-        <v>12</v>
-      </c>
-      <c r="E18" s="26" t="n">
-        <v>32</v>
-      </c>
-      <c r="F18" s="32" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G18" s="32" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="E18" s="26" t="n"/>
+      <c r="F18" s="32" t="n"/>
+      <c r="G18" s="32" t="n"/>
       <c r="H18" s="19" t="n">
         <v>1</v>
       </c>
@@ -4628,7 +4654,7 @@
         <v/>
       </c>
       <c r="K18" s="34">
-        <f>MIN(16,FLOOR(60*service_hr/J18,1))</f>
+        <f>MIN(10,FLOOR(60*service_hr/J18,1))</f>
         <v/>
       </c>
       <c r="L18" s="34">
@@ -4716,7 +4742,7 @@
         <v/>
       </c>
       <c r="AG18" s="31" t="n">
-        <v>344000</v>
+        <v>1750000</v>
       </c>
       <c r="AH18" s="32" t="n"/>
       <c r="AI18" s="32" t="n"/>
@@ -4759,161 +4785,378 @@
         <f>IF(((S18*pax_cap*load_full*ROUND(K18*L18*revleg_full,0))-(((battery/range_nm)*D18*ROUND(K18*L18*revleg_full,0)*VLOOKUP(B18,country_opex,3,FALSE))+V18+W18+X18+Y18+Z18))&lt;=0,"",VLOOKUP(B18,country_opex,7,FALSE)/((S18*pax_cap*load_full*ROUND(K18*L18*revleg_full,0))-(((battery/range_nm)*D18*ROUND(K18*L18*revleg_full,0)*VLOOKUP(B18,country_opex,3,FALSE))+V18+W18+X18+Y18+Z18)))</f>
         <v/>
       </c>
-      <c r="AW18" s="44" t="inlineStr">
+      <c r="AW18" s="44" t="n"/>
+      <c r="AX18" s="44" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>Yassir Tunisia</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>Sousse (Port El Kantaoui) → Monastir (Marina)</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="E19" s="26" t="n">
+        <v>32</v>
+      </c>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H19" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="33">
+        <f>60*D19/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J19" s="33">
+        <f>I19+turn_min+dwell_min</f>
+        <v/>
+      </c>
+      <c r="K19" s="34">
+        <f>MIN(16,FLOOR(60*service_hr/J19,1))</f>
+        <v/>
+      </c>
+      <c r="L19" s="34">
+        <f>ROUND(365*mech_uptime*H19,0)</f>
+        <v/>
+      </c>
+      <c r="M19" s="35">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="N19" s="35">
+        <f>revleg_sel</f>
+        <v/>
+      </c>
+      <c r="O19" s="34">
+        <f>ROUND(K19*L19*revleg_sel,0)</f>
+        <v/>
+      </c>
+      <c r="P19" s="36">
+        <f>load_sel</f>
+        <v/>
+      </c>
+      <c r="Q19" s="36">
+        <f>pax_cap*P19</f>
+        <v/>
+      </c>
+      <c r="R19" s="34">
+        <f>Q19*O19</f>
+        <v/>
+      </c>
+      <c r="S19" s="37">
+        <f>E19*discount</f>
+        <v/>
+      </c>
+      <c r="T19" s="38">
+        <f>S19*R19</f>
+        <v/>
+      </c>
+      <c r="U19" s="38">
+        <f>(battery/range_nm)*D19*O19*VLOOKUP(B19,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="V19" s="38">
+        <f>VLOOKUP(B19,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="W19" s="38">
+        <f>VLOOKUP(B19,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="X19" s="38">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Y19" s="38">
+        <f>VLOOKUP(B19,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="Z19" s="38">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AA19" s="38">
+        <f>U19+V19+W19+X19+Y19+Z19</f>
+        <v/>
+      </c>
+      <c r="AB19" s="38">
+        <f>VLOOKUP(B19,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AC19" s="38">
+        <f>T19-AA19</f>
+        <v/>
+      </c>
+      <c r="AD19" s="35">
+        <f>IF(T19=0,"",AC19/T19)</f>
+        <v/>
+      </c>
+      <c r="AE19" s="36">
+        <f>IF(AC19&lt;=0,"",VLOOKUP(B19,country_opex,7,FALSE)/AC19)</f>
+        <v/>
+      </c>
+      <c r="AF19" s="33">
+        <f>((D19*O19/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D19*O19*VLOOKUP(B19,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AG19" s="31" t="n">
+        <v>344000</v>
+      </c>
+      <c r="AH19" s="32" t="n"/>
+      <c r="AI19" s="32" t="n"/>
+      <c r="AJ19" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AK19" s="34">
+        <f>IF(AG19="","",AG19*AJ19)</f>
+        <v/>
+      </c>
+      <c r="AL19" s="34">
+        <f>IF(OR(AG19="",R19=0),"",MIN(IF(AS19="",9.9E+99,AS19),FLOOR(AK19/R19,1)))</f>
+        <v/>
+      </c>
+      <c r="AM19" s="38">
+        <f>IF(AL19="","",AL19*T19)</f>
+        <v/>
+      </c>
+      <c r="AN19" s="36">
+        <f>IF(OR(AG19="",R19=0),"",MIN(IF(AS19="",9.9E+99,AS19),AK19/R19))</f>
+        <v/>
+      </c>
+      <c r="AO19" s="38">
+        <f>IF(AN19="","",AN19*T19)</f>
+        <v/>
+      </c>
+      <c r="AP19" s="40" t="n"/>
+      <c r="AQ19" s="41" t="n"/>
+      <c r="AR19" s="41" t="n"/>
+      <c r="AS19" s="42" t="n"/>
+      <c r="AT19" s="43">
+        <f>IF(((S19*pax_cap*load_thin*ROUND(K19*L19*revleg_thin,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_thin,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19))&lt;=0,"",VLOOKUP(B19,country_opex,7,FALSE)/((S19*pax_cap*load_thin*ROUND(K19*L19*revleg_thin,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_thin,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19)))</f>
+        <v/>
+      </c>
+      <c r="AU19" s="43">
+        <f>IF(((S19*pax_cap*load_mid*ROUND(K19*L19*revleg_mid,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_mid,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19))&lt;=0,"",VLOOKUP(B19,country_opex,7,FALSE)/((S19*pax_cap*load_mid*ROUND(K19*L19*revleg_mid,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_mid,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19)))</f>
+        <v/>
+      </c>
+      <c r="AV19" s="43">
+        <f>IF(((S19*pax_cap*load_full*ROUND(K19*L19*revleg_full,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_full,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19))&lt;=0,"",VLOOKUP(B19,country_opex,7,FALSE)/((S19*pax_cap*load_full*ROUND(K19*L19*revleg_full,0))-(((battery/range_nm)*D19*ROUND(K19*L19*revleg_full,0)*VLOOKUP(B19,country_opex,3,FALSE))+V19+W19+X19+Y19+Z19)))</f>
+        <v/>
+      </c>
+      <c r="AW19" s="44" t="inlineStr">
         <is>
           <t>PREMIUM charter-divided tier: Port El Kantaoui per-seat catamaran / 'pirate boat' coastal cruise ~EUR 25-35 (Catamaran Amira day-cruise; half-day pirate-boat Sousse-Monastir) -&gt; midpoint ~EUR 30 x 1.08 ~= $32. This is the nearest premium per-seat water product operating on this exact coast.</t>
         </is>
       </c>
-      <c r="AX18" s="44" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="45" t="inlineStr">
+      <c r="AX19" s="44" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="45" t="inlineStr">
         <is>
           <t>TOTAL / median</t>
         </is>
       </c>
-      <c r="T19" s="46">
-        <f>SUM(T4:T18)</f>
-        <v/>
-      </c>
-      <c r="AC19" s="46">
-        <f>SUM(AC4:AC18)</f>
-        <v/>
-      </c>
-      <c r="AD19" s="47">
-        <f>IF(T19=0,"",AC19/T19)</f>
-        <v/>
-      </c>
-      <c r="AL19" s="48">
-        <f>SUM(AL4:AL18)</f>
-        <v/>
-      </c>
-      <c r="AM19" s="46">
-        <f>SUM(AM4:AM18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="T20" s="46">
+        <f>SUM(T4:T19)</f>
+        <v/>
+      </c>
+      <c r="AC20" s="46">
+        <f>SUM(AC4:AC19)</f>
+        <v/>
+      </c>
+      <c r="AD20" s="47">
+        <f>IF(T20=0,"",AC20/T20)</f>
+        <v/>
+      </c>
+      <c r="AL20" s="48">
+        <f>SUM(AL4:AL19)</f>
+        <v/>
+      </c>
+      <c r="AM20" s="46">
+        <f>SUM(AM4:AM19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Market fleet build-up — grounded floor (network-sum of raw vessel fractions per market, rounded once; subset slices excluded; legacy per-corridor-floor totals above kept for reference)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="24" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B23" s="24" t="inlineStr">
         <is>
           <t>Fleet basis</t>
         </is>
       </c>
-      <c r="C22" s="24" t="inlineStr">
+      <c r="C23" s="24" t="inlineStr">
         <is>
           <t>Raw vessels (sum)</t>
         </is>
       </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="D23" s="24" t="inlineStr">
         <is>
           <t>Fleet (rounded once)</t>
         </is>
       </c>
-      <c r="E22" s="24" t="inlineStr">
+      <c r="E23" s="24" t="inlineStr">
         <is>
           <t>Market rev/yr (raw sum)</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="25" t="inlineStr">
-        <is>
-          <t>Yassir Morocco</t>
-        </is>
-      </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>aspirational</t>
-        </is>
-      </c>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D23" s="49">
-        <f>SUMIFS(AL4:AL18,A4:A18,"Yassir Morocco",AP4:AP18,"=",AQ4:AQ18,"=",AR4:AR18,"=")</f>
-        <v/>
-      </c>
-      <c r="E23" s="50">
-        <f>SUMIFS(AM4:AM18,A4:A18,"Yassir Morocco",AP4:AP18,"=",AQ4:AQ18,"=",AR4:AR18,"=")</f>
-        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="25" t="inlineStr">
         <is>
+          <t>Yassir Algeria</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>aspirational</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D24" s="49">
+        <f>SUMIFS(AL4:AL19,A4:A19,"Yassir Algeria",AP4:AP19,"=",AQ4:AQ19,"=",AR4:AR19,"=")</f>
+        <v/>
+      </c>
+      <c r="E24" s="50">
+        <f>SUMIFS(AM4:AM19,A4:A19,"Yassir Algeria",AP4:AP19,"=",AQ4:AQ19,"=",AR4:AR19,"=")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>Yassir Morocco</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>aspirational</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D25" s="49">
+        <f>SUMIFS(AL4:AL19,A4:A19,"Yassir Morocco",AP4:AP19,"=",AQ4:AQ19,"=",AR4:AR19,"=")</f>
+        <v/>
+      </c>
+      <c r="E25" s="50">
+        <f>SUMIFS(AM4:AM19,A4:A19,"Yassir Morocco",AP4:AP19,"=",AQ4:AQ19,"=",AR4:AR19,"=")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
           <t>Yassir Tunisia</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>aspirational</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C26" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D24" s="49">
-        <f>SUMIFS(AL4:AL18,A4:A18,"Yassir Tunisia",AP4:AP18,"=",AQ4:AQ18,"=",AR4:AR18,"=")</f>
-        <v/>
-      </c>
-      <c r="E24" s="50">
-        <f>SUMIFS(AM4:AM18,A4:A18,"Yassir Tunisia",AP4:AP18,"=",AQ4:AQ18,"=",AR4:AR18,"=")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="45" t="inlineStr">
+      <c r="D26" s="49">
+        <f>SUMIFS(AL4:AL19,A4:A19,"Yassir Tunisia",AP4:AP19,"=",AQ4:AQ19,"=",AR4:AR19,"=")</f>
+        <v/>
+      </c>
+      <c r="E26" s="50">
+        <f>SUMIFS(AM4:AM19,A4:A19,"Yassir Tunisia",AP4:AP19,"=",AQ4:AQ19,"=",AR4:AR19,"=")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="45" t="inlineStr">
         <is>
           <t>GROUNDED FLOOR (PUBLISHED)</t>
         </is>
       </c>
-      <c r="D25" s="48">
-        <f>SUM(D23:D24)</f>
-        <v/>
-      </c>
-      <c r="E25" s="46">
-        <f>SUM(E23:E24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="51" t="inlineStr">
+      <c r="D27" s="48">
+        <f>SUM(D24:D26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="46">
+        <f>SUM(E24:E26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="51" t="inlineStr">
         <is>
           <t>Held for Quanta-LR (&gt;70nm, roadmap H2 2026+):</t>
         </is>
       </c>
-      <c r="C27" s="52" t="inlineStr">
+      <c r="C29" s="52" t="inlineStr">
         <is>
           <t>Tunis (La Goulette) → Palermo (Sicily, Italy) (170nm)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="C28" s="52" t="inlineStr">
+    <row r="30">
+      <c r="C30" s="52" t="inlineStr">
         <is>
           <t>Nador (Beni Ensar) → Almeria (Spain) (92nm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" s="52" t="inlineStr">
+        <is>
+          <t>Port d'Oran → Mostaganem port (81.7nm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" s="52" t="inlineStr">
+        <is>
+          <t>Port de Béjaïa → Port d'Alger (113.8nm)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A21:L21"/>
+    <mergeCell ref="A22:L22"/>
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5083,7 +5326,7 @@
         </is>
       </c>
       <c r="C11" s="39" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.09669999999999999</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>

</xml_diff>